<commit_message>
Fix match points calculation: use actual game scores as base points, not differential-based splits
</commit_message>
<xml_diff>
--- a/src/teams.xlsx
+++ b/src/teams.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7a2db4df0a309fda/Labs/ConcourCast/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="145" documentId="8_{C52A6B2E-3AE3-3848-B1F7-02D66D633EFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF2115C2-92DB-2149-82AA-5597A4761DFE}"/>
+  <xr:revisionPtr revIDLastSave="175" documentId="8_{C52A6B2E-3AE3-3848-B1F7-02D66D633EFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D18D0AC9-93F6-9B4A-A17D-401BD766CA59}"/>
   <bookViews>
     <workbookView xWindow="16180" yWindow="660" windowWidth="14060" windowHeight="17480" activeTab="1" xr2:uid="{76B42AAD-E78D-5C47-A529-CA0D1ECA81C5}"/>
   </bookViews>
@@ -1345,8 +1345,14 @@
       <c r="C32" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D32">
+        <v>7</v>
+      </c>
+      <c r="E32">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>3</v>
       </c>
@@ -1356,8 +1362,14 @@
       <c r="C33" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D33">
+        <v>3</v>
+      </c>
+      <c r="E33">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>3</v>
       </c>
@@ -1367,8 +1379,14 @@
       <c r="C34" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D34">
+        <v>9</v>
+      </c>
+      <c r="E34">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>3</v>
       </c>
@@ -1378,8 +1396,14 @@
       <c r="C35" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D35">
+        <v>7</v>
+      </c>
+      <c r="E35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>3</v>
       </c>
@@ -1389,8 +1413,14 @@
       <c r="C36" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D36">
+        <v>7</v>
+      </c>
+      <c r="E36">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>3</v>
       </c>
@@ -1400,8 +1430,14 @@
       <c r="C37" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D37">
+        <v>6</v>
+      </c>
+      <c r="E37">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>3</v>
       </c>
@@ -1411,8 +1447,14 @@
       <c r="C38" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D38">
+        <v>9</v>
+      </c>
+      <c r="E38">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>3</v>
       </c>
@@ -1422,8 +1464,14 @@
       <c r="C39" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D39">
+        <v>4</v>
+      </c>
+      <c r="E39">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>3</v>
       </c>
@@ -1433,8 +1481,14 @@
       <c r="C40" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>3</v>
       </c>
@@ -1444,8 +1498,14 @@
       <c r="C41" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D41">
+        <v>7</v>
+      </c>
+      <c r="E41">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>3</v>
       </c>
@@ -1455,8 +1515,14 @@
       <c r="C42" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D42">
+        <v>3</v>
+      </c>
+      <c r="E42">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>3</v>
       </c>
@@ -1466,8 +1532,14 @@
       <c r="C43" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D43">
+        <v>9</v>
+      </c>
+      <c r="E43">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>3</v>
       </c>
@@ -1477,8 +1549,14 @@
       <c r="C44" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D44">
+        <v>4</v>
+      </c>
+      <c r="E44">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>3</v>
       </c>
@@ -1488,8 +1566,14 @@
       <c r="C45" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D45">
+        <v>5</v>
+      </c>
+      <c r="E45">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>3</v>
       </c>
@@ -1499,8 +1583,14 @@
       <c r="C46" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D46">
+        <v>9</v>
+      </c>
+      <c r="E46">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>4</v>
       </c>
@@ -1511,7 +1601,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
fixed errors in excel
</commit_message>
<xml_diff>
--- a/src/teams.xlsx
+++ b/src/teams.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7a2db4df0a309fda/Labs/ConcourCast/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="175" documentId="8_{C52A6B2E-3AE3-3848-B1F7-02D66D633EFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D18D0AC9-93F6-9B4A-A17D-401BD766CA59}"/>
+  <xr:revisionPtr revIDLastSave="178" documentId="8_{C52A6B2E-3AE3-3848-B1F7-02D66D633EFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E013B543-3FB4-1C4A-B9F1-FB0F6A99E169}"/>
   <bookViews>
     <workbookView xWindow="16180" yWindow="660" windowWidth="14060" windowHeight="17480" activeTab="1" xr2:uid="{76B42AAD-E78D-5C47-A529-CA0D1ECA81C5}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="42">
   <si>
     <t>TeamName</t>
   </si>
@@ -163,9 +163,6 @@
   </si>
   <si>
     <t>B</t>
-  </si>
-  <si>
-    <t>Dublin</t>
   </si>
 </sst>
 </file>
@@ -1326,7 +1323,7 @@
         <v>6</v>
       </c>
       <c r="C31" t="s">
-        <v>42</v>
+        <v>7</v>
       </c>
       <c r="D31">
         <v>4</v>
@@ -1374,7 +1371,7 @@
         <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C34" t="s">
         <v>26</v>
@@ -1620,7 +1617,7 @@
         <v>24</v>
       </c>
       <c r="C49" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>